<commit_message>
added detailed trim info to recap
</commit_message>
<xml_diff>
--- a/CustomLabelPrinter/src/paperwork/dsi/recap.xlsx
+++ b/CustomLabelPrinter/src/paperwork/dsi/recap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\git\CustomLabelPrinter\CustomLabelPrinter\src\paperwork\dsi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3A54D9F-7807-4FC8-B5B0-3AE2EA2AB64A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9CE39E2-5E4A-480F-934A-EB1FB7DB8BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="615" yWindow="2310" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BREAST" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="42">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -149,6 +149,15 @@
   </si>
   <si>
     <t>DSI Condemned</t>
+  </si>
+  <si>
+    <t>Table</t>
+  </si>
+  <si>
+    <t>Trimming weights:</t>
+  </si>
+  <si>
+    <t>DSI</t>
   </si>
 </sst>
 </file>
@@ -570,7 +579,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -664,6 +673,9 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -676,6 +688,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -688,11 +706,59 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -718,65 +784,14 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -784,11 +799,8 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1082,54 +1094,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:19" ht="35.25" x14ac:dyDescent="0.25">
-      <c r="C1" s="45" t="s">
+      <c r="C1" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="45"/>
-      <c r="N1" s="45"/>
-      <c r="O1" s="45"/>
-      <c r="P1" s="45"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
+      <c r="P1" s="46"/>
     </row>
     <row r="2" spans="2:19" ht="27.75" x14ac:dyDescent="0.4">
       <c r="C2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="46"/>
-      <c r="F2" s="47" t="s">
+      <c r="E2" s="47"/>
+      <c r="F2" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
       <c r="L2" s="7"/>
       <c r="M2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
       <c r="P2" s="7"/>
     </row>
     <row r="3" spans="2:19" s="1" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
     </row>
     <row r="4" spans="2:19" s="1" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E4" s="8">
@@ -1162,10 +1174,10 @@
       <c r="N4" s="8">
         <v>26</v>
       </c>
-      <c r="O4" s="48" t="s">
+      <c r="O4" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="P4" s="48"/>
+      <c r="P4" s="49"/>
       <c r="R4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1961,57 +1973,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:19" ht="35.25" x14ac:dyDescent="0.25">
-      <c r="C1" s="45" t="s">
+      <c r="C1" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="45"/>
-      <c r="N1" s="45"/>
-      <c r="O1" s="45"/>
-      <c r="P1" s="45"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
+      <c r="P1" s="46"/>
     </row>
     <row r="2" spans="2:19" ht="27.75" x14ac:dyDescent="0.4">
       <c r="C2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="46"/>
-      <c r="F2" s="47" t="s">
+      <c r="E2" s="47"/>
+      <c r="F2" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
       <c r="L2" s="7"/>
       <c r="M2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
       <c r="P2" s="7"/>
       <c r="S2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="2:19" s="1" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
     </row>
     <row r="4" spans="2:19" s="1" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E4" s="8">
@@ -2044,10 +2056,10 @@
       <c r="N4" s="8">
         <v>26</v>
       </c>
-      <c r="O4" s="48" t="s">
+      <c r="O4" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="P4" s="48"/>
+      <c r="P4" s="49"/>
     </row>
     <row r="5" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="15"/>
@@ -2837,54 +2849,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:19" ht="35.25" x14ac:dyDescent="0.25">
-      <c r="C1" s="45" t="s">
+      <c r="C1" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="45"/>
-      <c r="N1" s="45"/>
-      <c r="O1" s="45"/>
-      <c r="P1" s="45"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
+      <c r="P1" s="46"/>
     </row>
     <row r="2" spans="2:19" ht="27.75" x14ac:dyDescent="0.4">
       <c r="C2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="46"/>
-      <c r="F2" s="47" t="s">
+      <c r="E2" s="47"/>
+      <c r="F2" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
       <c r="L2" s="7"/>
       <c r="M2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
       <c r="P2" s="7"/>
     </row>
     <row r="3" spans="2:19" s="1" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
     </row>
     <row r="4" spans="2:19" s="1" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E4" s="8">
@@ -2917,20 +2929,20 @@
       <c r="N4" s="8">
         <v>26</v>
       </c>
-      <c r="O4" s="48" t="s">
+      <c r="O4" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="P4" s="48"/>
+      <c r="P4" s="49"/>
       <c r="S4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="15"/>
-      <c r="C5" s="53">
+      <c r="C5" s="50">
         <v>21102</v>
       </c>
-      <c r="D5" s="54"/>
+      <c r="D5" s="51"/>
       <c r="E5" s="16"/>
       <c r="F5" s="17"/>
       <c r="G5" s="17"/>
@@ -2941,13 +2953,13 @@
       <c r="L5" s="17"/>
       <c r="M5" s="17"/>
       <c r="N5" s="18"/>
-      <c r="O5" s="55"/>
-      <c r="P5" s="56"/>
+      <c r="O5" s="74"/>
+      <c r="P5" s="75"/>
     </row>
     <row r="6" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="15"/>
-      <c r="C6" s="49"/>
-      <c r="D6" s="50"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="53"/>
       <c r="E6" s="19"/>
       <c r="F6" s="20"/>
       <c r="G6" s="20"/>
@@ -2958,13 +2970,13 @@
       <c r="L6" s="20"/>
       <c r="M6" s="20"/>
       <c r="N6" s="21"/>
-      <c r="O6" s="57"/>
-      <c r="P6" s="58"/>
+      <c r="O6" s="76"/>
+      <c r="P6" s="77"/>
     </row>
     <row r="7" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="15"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="50"/>
+      <c r="C7" s="52"/>
+      <c r="D7" s="53"/>
       <c r="E7" s="19"/>
       <c r="F7" s="20"/>
       <c r="G7" s="20"/>
@@ -2975,13 +2987,13 @@
       <c r="L7" s="20"/>
       <c r="M7" s="20"/>
       <c r="N7" s="21"/>
-      <c r="O7" s="59"/>
-      <c r="P7" s="60"/>
+      <c r="O7" s="78"/>
+      <c r="P7" s="79"/>
     </row>
     <row r="8" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="15"/>
-      <c r="C8" s="49"/>
-      <c r="D8" s="50"/>
+      <c r="C8" s="52"/>
+      <c r="D8" s="53"/>
       <c r="E8" s="19"/>
       <c r="F8" s="20"/>
       <c r="G8" s="20"/>
@@ -2992,13 +3004,13 @@
       <c r="L8" s="20"/>
       <c r="M8" s="20"/>
       <c r="N8" s="21"/>
-      <c r="O8" s="59"/>
-      <c r="P8" s="60"/>
+      <c r="O8" s="78"/>
+      <c r="P8" s="79"/>
     </row>
     <row r="9" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="15"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="50"/>
+      <c r="C9" s="52"/>
+      <c r="D9" s="53"/>
       <c r="E9" s="19"/>
       <c r="F9" s="20"/>
       <c r="G9" s="20"/>
@@ -3009,13 +3021,13 @@
       <c r="L9" s="20"/>
       <c r="M9" s="20"/>
       <c r="N9" s="21"/>
-      <c r="O9" s="59"/>
-      <c r="P9" s="60"/>
+      <c r="O9" s="78"/>
+      <c r="P9" s="79"/>
     </row>
     <row r="10" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="15"/>
-      <c r="C10" s="49"/>
-      <c r="D10" s="50"/>
+      <c r="C10" s="52"/>
+      <c r="D10" s="53"/>
       <c r="E10" s="19"/>
       <c r="F10" s="20"/>
       <c r="G10" s="20"/>
@@ -3026,13 +3038,13 @@
       <c r="L10" s="20"/>
       <c r="M10" s="20"/>
       <c r="N10" s="21"/>
-      <c r="O10" s="59"/>
-      <c r="P10" s="60"/>
+      <c r="O10" s="78"/>
+      <c r="P10" s="79"/>
     </row>
     <row r="11" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="15"/>
-      <c r="C11" s="49"/>
-      <c r="D11" s="50"/>
+      <c r="C11" s="52"/>
+      <c r="D11" s="53"/>
       <c r="E11" s="19"/>
       <c r="F11" s="20"/>
       <c r="G11" s="20"/>
@@ -3043,13 +3055,13 @@
       <c r="L11" s="20"/>
       <c r="M11" s="20"/>
       <c r="N11" s="21"/>
-      <c r="O11" s="59"/>
-      <c r="P11" s="60"/>
+      <c r="O11" s="78"/>
+      <c r="P11" s="79"/>
     </row>
     <row r="12" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="15"/>
-      <c r="C12" s="49"/>
-      <c r="D12" s="50"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="53"/>
       <c r="E12" s="19"/>
       <c r="F12" s="20"/>
       <c r="G12" s="20"/>
@@ -3060,13 +3072,13 @@
       <c r="L12" s="20"/>
       <c r="M12" s="20"/>
       <c r="N12" s="21"/>
-      <c r="O12" s="59"/>
-      <c r="P12" s="60"/>
+      <c r="O12" s="78"/>
+      <c r="P12" s="79"/>
     </row>
     <row r="13" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="15"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="50"/>
+      <c r="C13" s="52"/>
+      <c r="D13" s="53"/>
       <c r="E13" s="19"/>
       <c r="F13" s="20"/>
       <c r="G13" s="20"/>
@@ -3077,13 +3089,13 @@
       <c r="L13" s="20"/>
       <c r="M13" s="20"/>
       <c r="N13" s="21"/>
-      <c r="O13" s="59"/>
-      <c r="P13" s="60"/>
+      <c r="O13" s="78"/>
+      <c r="P13" s="79"/>
     </row>
     <row r="14" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="15"/>
-      <c r="C14" s="49"/>
-      <c r="D14" s="50"/>
+      <c r="C14" s="52"/>
+      <c r="D14" s="53"/>
       <c r="E14" s="19"/>
       <c r="F14" s="20"/>
       <c r="G14" s="20"/>
@@ -3094,13 +3106,13 @@
       <c r="L14" s="20"/>
       <c r="M14" s="20"/>
       <c r="N14" s="21"/>
-      <c r="O14" s="59"/>
-      <c r="P14" s="60"/>
+      <c r="O14" s="78"/>
+      <c r="P14" s="79"/>
     </row>
     <row r="15" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="15"/>
-      <c r="C15" s="49"/>
-      <c r="D15" s="50"/>
+      <c r="C15" s="52"/>
+      <c r="D15" s="53"/>
       <c r="E15" s="19"/>
       <c r="F15" s="20"/>
       <c r="G15" s="20"/>
@@ -3113,13 +3125,13 @@
       <c r="L15" s="20"/>
       <c r="M15" s="20"/>
       <c r="N15" s="21"/>
-      <c r="O15" s="59"/>
-      <c r="P15" s="60"/>
+      <c r="O15" s="78"/>
+      <c r="P15" s="79"/>
     </row>
     <row r="16" spans="2:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="15"/>
-      <c r="C16" s="49"/>
-      <c r="D16" s="50"/>
+      <c r="C16" s="52"/>
+      <c r="D16" s="53"/>
       <c r="E16" s="19"/>
       <c r="F16" s="20"/>
       <c r="G16" s="20"/>
@@ -3130,13 +3142,13 @@
       <c r="L16" s="20"/>
       <c r="M16" s="20"/>
       <c r="N16" s="21"/>
-      <c r="O16" s="59"/>
-      <c r="P16" s="60"/>
+      <c r="O16" s="78"/>
+      <c r="P16" s="79"/>
     </row>
     <row r="17" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="15"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="50"/>
+      <c r="C17" s="52"/>
+      <c r="D17" s="53"/>
       <c r="E17" s="22"/>
       <c r="F17" s="23"/>
       <c r="G17" s="23"/>
@@ -3147,13 +3159,13 @@
       <c r="L17" s="23"/>
       <c r="M17" s="23"/>
       <c r="N17" s="24"/>
-      <c r="O17" s="59"/>
-      <c r="P17" s="60"/>
+      <c r="O17" s="78"/>
+      <c r="P17" s="79"/>
     </row>
     <row r="18" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="15"/>
-      <c r="C18" s="49"/>
-      <c r="D18" s="50"/>
+      <c r="C18" s="52"/>
+      <c r="D18" s="53"/>
       <c r="E18" s="11"/>
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
@@ -3164,13 +3176,13 @@
       <c r="L18" s="9"/>
       <c r="M18" s="9"/>
       <c r="N18" s="12"/>
-      <c r="O18" s="59"/>
-      <c r="P18" s="60"/>
+      <c r="O18" s="78"/>
+      <c r="P18" s="79"/>
     </row>
     <row r="19" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="15"/>
-      <c r="C19" s="49"/>
-      <c r="D19" s="50"/>
+      <c r="C19" s="52"/>
+      <c r="D19" s="53"/>
       <c r="E19" s="11"/>
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
@@ -3181,13 +3193,13 @@
       <c r="L19" s="9"/>
       <c r="M19" s="9"/>
       <c r="N19" s="12"/>
-      <c r="O19" s="59"/>
-      <c r="P19" s="60"/>
+      <c r="O19" s="78"/>
+      <c r="P19" s="79"/>
     </row>
     <row r="20" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="15"/>
-      <c r="C20" s="49"/>
-      <c r="D20" s="50"/>
+      <c r="C20" s="52"/>
+      <c r="D20" s="53"/>
       <c r="E20" s="11"/>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
@@ -3198,13 +3210,13 @@
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
       <c r="N20" s="12"/>
-      <c r="O20" s="59"/>
-      <c r="P20" s="60"/>
+      <c r="O20" s="78"/>
+      <c r="P20" s="79"/>
     </row>
     <row r="21" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="15"/>
-      <c r="C21" s="49"/>
-      <c r="D21" s="50"/>
+      <c r="C21" s="52"/>
+      <c r="D21" s="53"/>
       <c r="E21" s="11"/>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
@@ -3215,13 +3227,13 @@
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
       <c r="N21" s="12"/>
-      <c r="O21" s="59"/>
-      <c r="P21" s="60"/>
+      <c r="O21" s="78"/>
+      <c r="P21" s="79"/>
     </row>
     <row r="22" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="15"/>
-      <c r="C22" s="49"/>
-      <c r="D22" s="50"/>
+      <c r="C22" s="52"/>
+      <c r="D22" s="53"/>
       <c r="E22" s="11"/>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
@@ -3232,13 +3244,13 @@
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
       <c r="N22" s="12"/>
-      <c r="O22" s="59"/>
-      <c r="P22" s="60"/>
+      <c r="O22" s="78"/>
+      <c r="P22" s="79"/>
     </row>
     <row r="23" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="15"/>
-      <c r="C23" s="49"/>
-      <c r="D23" s="50"/>
+      <c r="C23" s="52"/>
+      <c r="D23" s="53"/>
       <c r="E23" s="11"/>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
@@ -3249,13 +3261,13 @@
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="12"/>
-      <c r="O23" s="59"/>
-      <c r="P23" s="60"/>
+      <c r="O23" s="78"/>
+      <c r="P23" s="79"/>
     </row>
     <row r="24" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="15"/>
-      <c r="C24" s="49"/>
-      <c r="D24" s="50"/>
+      <c r="C24" s="52"/>
+      <c r="D24" s="53"/>
       <c r="E24" s="11"/>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
@@ -3266,13 +3278,13 @@
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="12"/>
-      <c r="O24" s="59"/>
-      <c r="P24" s="60"/>
+      <c r="O24" s="78"/>
+      <c r="P24" s="79"/>
     </row>
     <row r="25" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="15"/>
-      <c r="C25" s="49"/>
-      <c r="D25" s="50"/>
+      <c r="C25" s="52"/>
+      <c r="D25" s="53"/>
       <c r="E25" s="11"/>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -3283,13 +3295,13 @@
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="12"/>
-      <c r="O25" s="59"/>
-      <c r="P25" s="60"/>
+      <c r="O25" s="78"/>
+      <c r="P25" s="79"/>
     </row>
     <row r="26" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="15"/>
-      <c r="C26" s="49"/>
-      <c r="D26" s="50"/>
+      <c r="C26" s="52"/>
+      <c r="D26" s="53"/>
       <c r="E26" s="11"/>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
@@ -3300,13 +3312,13 @@
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="12"/>
-      <c r="O26" s="59"/>
-      <c r="P26" s="60"/>
+      <c r="O26" s="78"/>
+      <c r="P26" s="79"/>
     </row>
     <row r="27" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B27" s="15"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="52"/>
+      <c r="C27" s="54"/>
+      <c r="D27" s="55"/>
       <c r="E27" s="4"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -3317,13 +3329,13 @@
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
       <c r="N27" s="13"/>
-      <c r="O27" s="61"/>
-      <c r="P27" s="62"/>
+      <c r="O27" s="80"/>
+      <c r="P27" s="81"/>
     </row>
     <row r="28" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="15"/>
-      <c r="C28" s="53"/>
-      <c r="D28" s="54"/>
+      <c r="C28" s="50"/>
+      <c r="D28" s="51"/>
       <c r="E28" s="6"/>
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
@@ -3334,13 +3346,13 @@
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
       <c r="N28" s="10"/>
-      <c r="O28" s="63"/>
-      <c r="P28" s="64"/>
+      <c r="O28" s="56"/>
+      <c r="P28" s="57"/>
     </row>
     <row r="29" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="15"/>
-      <c r="C29" s="49"/>
-      <c r="D29" s="50"/>
+      <c r="C29" s="52"/>
+      <c r="D29" s="53"/>
       <c r="E29" s="11"/>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
@@ -3351,13 +3363,13 @@
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="12"/>
-      <c r="O29" s="65"/>
-      <c r="P29" s="66"/>
+      <c r="O29" s="58"/>
+      <c r="P29" s="59"/>
     </row>
     <row r="30" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="15"/>
-      <c r="C30" s="49"/>
-      <c r="D30" s="50"/>
+      <c r="C30" s="52"/>
+      <c r="D30" s="53"/>
       <c r="E30" s="11"/>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
@@ -3368,13 +3380,13 @@
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="12"/>
-      <c r="O30" s="65"/>
-      <c r="P30" s="66"/>
+      <c r="O30" s="58"/>
+      <c r="P30" s="59"/>
     </row>
     <row r="31" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="15"/>
-      <c r="C31" s="49"/>
-      <c r="D31" s="50"/>
+      <c r="C31" s="52"/>
+      <c r="D31" s="53"/>
       <c r="E31" s="11"/>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
@@ -3385,13 +3397,13 @@
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="12"/>
-      <c r="O31" s="65"/>
-      <c r="P31" s="66"/>
+      <c r="O31" s="58"/>
+      <c r="P31" s="59"/>
     </row>
     <row r="32" spans="2:16" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="15"/>
-      <c r="C32" s="49"/>
-      <c r="D32" s="50"/>
+      <c r="C32" s="52"/>
+      <c r="D32" s="53"/>
       <c r="E32" s="11"/>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
@@ -3402,13 +3414,13 @@
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="12"/>
-      <c r="O32" s="65"/>
-      <c r="P32" s="66"/>
+      <c r="O32" s="58"/>
+      <c r="P32" s="59"/>
     </row>
     <row r="33" spans="1:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="15"/>
-      <c r="C33" s="49"/>
-      <c r="D33" s="50"/>
+      <c r="C33" s="52"/>
+      <c r="D33" s="53"/>
       <c r="E33" s="11"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -3419,13 +3431,13 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="12"/>
-      <c r="O33" s="65"/>
-      <c r="P33" s="66"/>
+      <c r="O33" s="58"/>
+      <c r="P33" s="59"/>
     </row>
     <row r="34" spans="1:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="15"/>
-      <c r="C34" s="49"/>
-      <c r="D34" s="50"/>
+      <c r="C34" s="52"/>
+      <c r="D34" s="53"/>
       <c r="E34" s="11"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -3436,13 +3448,13 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="12"/>
-      <c r="O34" s="65"/>
-      <c r="P34" s="66"/>
+      <c r="O34" s="58"/>
+      <c r="P34" s="59"/>
     </row>
     <row r="35" spans="1:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="15"/>
-      <c r="C35" s="49"/>
-      <c r="D35" s="50"/>
+      <c r="C35" s="52"/>
+      <c r="D35" s="53"/>
       <c r="E35" s="11"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -3453,13 +3465,13 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="12"/>
-      <c r="O35" s="65"/>
-      <c r="P35" s="66"/>
+      <c r="O35" s="58"/>
+      <c r="P35" s="59"/>
     </row>
     <row r="36" spans="1:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="15"/>
-      <c r="C36" s="49"/>
-      <c r="D36" s="50"/>
+      <c r="C36" s="52"/>
+      <c r="D36" s="53"/>
       <c r="E36" s="11"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -3470,13 +3482,13 @@
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="12"/>
-      <c r="O36" s="65"/>
-      <c r="P36" s="66"/>
+      <c r="O36" s="58"/>
+      <c r="P36" s="59"/>
     </row>
     <row r="37" spans="1:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="15"/>
-      <c r="C37" s="49"/>
-      <c r="D37" s="50"/>
+      <c r="C37" s="52"/>
+      <c r="D37" s="53"/>
       <c r="E37" s="11"/>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -3487,13 +3499,13 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="12"/>
-      <c r="O37" s="65"/>
-      <c r="P37" s="66"/>
+      <c r="O37" s="58"/>
+      <c r="P37" s="59"/>
     </row>
     <row r="38" spans="1:19" s="1" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B38" s="15"/>
-      <c r="C38" s="51"/>
-      <c r="D38" s="52"/>
+      <c r="C38" s="54"/>
+      <c r="D38" s="55"/>
       <c r="E38" s="25"/>
       <c r="F38" s="26"/>
       <c r="G38" s="26"/>
@@ -3504,16 +3516,16 @@
       <c r="L38" s="26"/>
       <c r="M38" s="26"/>
       <c r="N38" s="27"/>
-      <c r="O38" s="67"/>
-      <c r="P38" s="68"/>
+      <c r="O38" s="60"/>
+      <c r="P38" s="61"/>
     </row>
     <row r="39" spans="1:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39"/>
       <c r="B39"/>
-      <c r="C39" s="69">
+      <c r="C39" s="62">
         <v>10468</v>
       </c>
-      <c r="D39" s="70"/>
+      <c r="D39" s="63"/>
       <c r="E39" s="42"/>
       <c r="F39" s="43"/>
       <c r="G39" s="43"/>
@@ -3524,8 +3536,8 @@
       <c r="L39" s="43"/>
       <c r="M39" s="43"/>
       <c r="N39" s="44"/>
-      <c r="O39" s="75"/>
-      <c r="P39" s="76"/>
+      <c r="O39" s="68"/>
+      <c r="P39" s="69"/>
       <c r="Q39"/>
       <c r="R39"/>
       <c r="S39"/>
@@ -3533,8 +3545,8 @@
     <row r="40" spans="1:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40"/>
       <c r="B40"/>
-      <c r="C40" s="71"/>
-      <c r="D40" s="72"/>
+      <c r="C40" s="64"/>
+      <c r="D40" s="65"/>
       <c r="E40" s="42"/>
       <c r="F40" s="43"/>
       <c r="G40" s="43"/>
@@ -3545,8 +3557,8 @@
       <c r="L40" s="43"/>
       <c r="M40" s="43"/>
       <c r="N40" s="44"/>
-      <c r="O40" s="77"/>
-      <c r="P40" s="78"/>
+      <c r="O40" s="70"/>
+      <c r="P40" s="71"/>
       <c r="Q40"/>
       <c r="R40"/>
       <c r="S40"/>
@@ -3554,8 +3566,8 @@
     <row r="41" spans="1:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41"/>
       <c r="B41"/>
-      <c r="C41" s="71"/>
-      <c r="D41" s="72"/>
+      <c r="C41" s="64"/>
+      <c r="D41" s="65"/>
       <c r="E41" s="42"/>
       <c r="F41" s="43"/>
       <c r="G41" s="43"/>
@@ -3566,8 +3578,8 @@
       <c r="L41" s="43"/>
       <c r="M41" s="43"/>
       <c r="N41" s="44"/>
-      <c r="O41" s="77"/>
-      <c r="P41" s="78"/>
+      <c r="O41" s="70"/>
+      <c r="P41" s="71"/>
       <c r="Q41"/>
       <c r="R41"/>
       <c r="S41"/>
@@ -3575,8 +3587,8 @@
     <row r="42" spans="1:19" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42"/>
       <c r="B42"/>
-      <c r="C42" s="71"/>
-      <c r="D42" s="72"/>
+      <c r="C42" s="64"/>
+      <c r="D42" s="65"/>
       <c r="E42" s="42"/>
       <c r="F42" s="43"/>
       <c r="G42" s="43"/>
@@ -3587,8 +3599,8 @@
       <c r="L42" s="43"/>
       <c r="M42" s="43"/>
       <c r="N42" s="44"/>
-      <c r="O42" s="77"/>
-      <c r="P42" s="78"/>
+      <c r="O42" s="70"/>
+      <c r="P42" s="71"/>
       <c r="Q42"/>
       <c r="R42"/>
       <c r="S42"/>
@@ -3596,8 +3608,8 @@
     <row r="43" spans="1:19" s="1" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43"/>
       <c r="B43"/>
-      <c r="C43" s="73"/>
-      <c r="D43" s="74"/>
+      <c r="C43" s="66"/>
+      <c r="D43" s="67"/>
       <c r="E43" s="42"/>
       <c r="F43" s="43"/>
       <c r="G43" s="43"/>
@@ -3608,8 +3620,8 @@
       <c r="L43" s="43"/>
       <c r="M43" s="43"/>
       <c r="N43" s="44"/>
-      <c r="O43" s="79"/>
-      <c r="P43" s="80"/>
+      <c r="O43" s="72"/>
+      <c r="P43" s="73"/>
       <c r="Q43"/>
       <c r="R43"/>
       <c r="S43"/>
@@ -3742,11 +3754,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="C28:D29"/>
-    <mergeCell ref="C30:D38"/>
-    <mergeCell ref="O28:P38"/>
-    <mergeCell ref="C39:D43"/>
-    <mergeCell ref="O39:P43"/>
     <mergeCell ref="C1:P1"/>
     <mergeCell ref="F2:K3"/>
     <mergeCell ref="N2:O2"/>
@@ -3756,6 +3763,11 @@
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="O5:P6"/>
     <mergeCell ref="O7:P27"/>
+    <mergeCell ref="C28:D29"/>
+    <mergeCell ref="C30:D38"/>
+    <mergeCell ref="O28:P38"/>
+    <mergeCell ref="C39:D43"/>
+    <mergeCell ref="O39:P43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="35" orientation="portrait" r:id="rId1"/>
@@ -4000,11 +4012,39 @@
       <c r="A31" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="B31" s="81"/>
-      <c r="C31" s="81"/>
+      <c r="B31" s="83"/>
+      <c r="C31" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A25:B26"/>
+    <mergeCell ref="C25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:G26"/>
+    <mergeCell ref="H25:I26"/>
+    <mergeCell ref="A27:B28"/>
+    <mergeCell ref="C27:D28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:G28"/>
+    <mergeCell ref="H27:I28"/>
+    <mergeCell ref="F19:G20"/>
+    <mergeCell ref="H19:I20"/>
+    <mergeCell ref="A17:B18"/>
+    <mergeCell ref="C17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:G18"/>
+    <mergeCell ref="H17:I18"/>
+    <mergeCell ref="A21:B22"/>
+    <mergeCell ref="C21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:G22"/>
+    <mergeCell ref="H21:I22"/>
+    <mergeCell ref="A23:B24"/>
+    <mergeCell ref="C23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:G24"/>
+    <mergeCell ref="H23:I24"/>
     <mergeCell ref="F13:G14"/>
     <mergeCell ref="H13:I14"/>
     <mergeCell ref="A15:B16"/>
@@ -4015,34 +4055,6 @@
     <mergeCell ref="A13:B14"/>
     <mergeCell ref="C13:D14"/>
     <mergeCell ref="E13:E14"/>
-    <mergeCell ref="A23:B24"/>
-    <mergeCell ref="C23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:G24"/>
-    <mergeCell ref="H23:I24"/>
-    <mergeCell ref="A21:B22"/>
-    <mergeCell ref="C21:D22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:G22"/>
-    <mergeCell ref="H21:I22"/>
-    <mergeCell ref="F19:G20"/>
-    <mergeCell ref="H19:I20"/>
-    <mergeCell ref="A17:B18"/>
-    <mergeCell ref="C17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:G18"/>
-    <mergeCell ref="H17:I18"/>
-    <mergeCell ref="H25:I26"/>
-    <mergeCell ref="A27:B28"/>
-    <mergeCell ref="C27:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:G28"/>
-    <mergeCell ref="H27:I28"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="A25:B26"/>
-    <mergeCell ref="C25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:G26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -4063,15 +4075,15 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="A3" s="83" t="s">
+      <c r="A3" s="85" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="83"/>
-      <c r="G3" s="83" t="s">
+      <c r="B3" s="85"/>
+      <c r="G3" s="85" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="83"/>
-      <c r="I3" s="83"/>
+      <c r="H3" s="85"/>
+      <c r="I3" s="85"/>
     </row>
     <row r="5" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G5" s="41" t="s">
@@ -4086,16 +4098,16 @@
       </c>
       <c r="B6" s="39"/>
       <c r="C6" s="36"/>
-      <c r="G6" s="84"/>
-      <c r="H6" s="84"/>
-      <c r="I6" s="84"/>
+      <c r="G6" s="86"/>
+      <c r="H6" s="86"/>
+      <c r="I6" s="86"/>
     </row>
     <row r="7" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="39"/>
       <c r="C7" s="36"/>
-      <c r="G7" s="84"/>
-      <c r="H7" s="84"/>
-      <c r="I7" s="84"/>
+      <c r="G7" s="86"/>
+      <c r="H7" s="86"/>
+      <c r="I7" s="86"/>
     </row>
     <row r="8" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="37"/>
@@ -4115,9 +4127,11 @@
     <row r="10" spans="1:9" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B10" s="39"/>
       <c r="C10" s="36"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="41"/>
-      <c r="I10" s="41"/>
+      <c r="G10" s="87" t="s">
+        <v>40</v>
+      </c>
+      <c r="H10" s="87"/>
+      <c r="I10" s="87"/>
     </row>
     <row r="11" spans="1:9" ht="18" x14ac:dyDescent="0.25">
       <c r="A11" s="37" t="s">
@@ -4125,9 +4139,13 @@
       </c>
       <c r="B11" s="39"/>
       <c r="C11" s="36"/>
-      <c r="G11" s="41"/>
+      <c r="G11" s="41" t="s">
+        <v>41</v>
+      </c>
       <c r="H11" s="41"/>
-      <c r="I11" s="41"/>
+      <c r="I11" s="41" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B12" s="39"/>
@@ -4151,7 +4169,7 @@
       </c>
       <c r="B16" s="39"/>
       <c r="C16" s="36"/>
-      <c r="G16" s="86" t="s">
+      <c r="G16" s="45" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4181,11 +4199,11 @@
     <row r="22" spans="1:9" ht="18" x14ac:dyDescent="0.25">
       <c r="B22" s="39"/>
       <c r="C22" s="36"/>
-      <c r="G22" s="83" t="s">
+      <c r="G22" s="85" t="s">
         <v>31</v>
       </c>
-      <c r="H22" s="83"/>
-      <c r="I22" s="83"/>
+      <c r="H22" s="85"/>
+      <c r="I22" s="85"/>
     </row>
     <row r="23" spans="1:9" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B23" s="39"/>
@@ -4304,11 +4322,11 @@
     <row r="39" spans="1:9" ht="18" x14ac:dyDescent="0.25">
       <c r="B39" s="39"/>
       <c r="C39" s="36"/>
-      <c r="G39" s="85" t="s">
+      <c r="G39" s="84" t="s">
         <v>38</v>
       </c>
-      <c r="H39" s="85"/>
-      <c r="I39" s="85"/>
+      <c r="H39" s="84"/>
+      <c r="I39" s="84"/>
     </row>
     <row r="40" spans="1:9" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B40" s="39"/>
@@ -4340,13 +4358,14 @@
       <c r="C45" s="36"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="G39:I39"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="G3:I3"/>
     <mergeCell ref="G22:I22"/>
     <mergeCell ref="G6:I6"/>
     <mergeCell ref="G7:I7"/>
+    <mergeCell ref="G10:I10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>